<commit_message>
Fix stage evidence types for the 12-step plan, show Tradio evidence in stage modal, no overdue on delivered, compact Kriyaa list_orders, seed data fixes
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/backend/src/db/demo-docs/measurements-baggy-active-jacket.xlsx
+++ b/backend/src/db/demo-docs/measurements-baggy-active-jacket.xlsx
@@ -663,7 +663,7 @@
         <v>56</v>
       </c>
       <c r="F12" s="5" t="n">
-        <v>69.5</v>
+        <v>59</v>
       </c>
       <c r="G12" s="5" t="n">
         <v>62</v>
@@ -695,7 +695,7 @@
         <v>56</v>
       </c>
       <c r="F13" s="5" t="n">
-        <v>69.5</v>
+        <v>59</v>
       </c>
       <c r="G13" s="5" t="n">
         <v>62</v>
@@ -845,19 +845,22 @@
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>24</t>
+          <t>±0.5</t>
         </is>
       </c>
       <c r="D18" s="5" t="n">
+        <v>24.5</v>
+      </c>
+      <c r="E18" s="5" t="n">
         <v>25.5</v>
       </c>
-      <c r="E18" s="5" t="n">
+      <c r="F18" s="5" t="n">
         <v>26.5</v>
       </c>
-      <c r="F18" s="5" t="n">
+      <c r="G18" s="5" t="n">
         <v>27.5</v>
       </c>
-      <c r="G18" s="5" t="n">
+      <c r="H18" s="5" t="n">
         <v>28.5</v>
       </c>
     </row>

</xml_diff>